<commit_message>
feat: Score champion selection in the poster rubric (M09/M10)
Criterion 6 becomes Model Comparison and Champion Selection: margin
with its business meaning and a simplest-first order stated before
comparing, the fold-corrected paired interval read as one of four
outcomes, and one champion justified in the stakeholder's terms.
Criterion 5 asks for fold scores with mean and SD, not a per-model
confidence interval. Transition notes keep M09 feedback-only and
protect nb08/nb14-style work and disclosed after-the-fact margins.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_final_project/2026F/rubric/Predictive_Analytics_Poster_Rubric.xlsx
+++ b/_final_project/2026F/rubric/Predictive_Analytics_Poster_Rubric.xlsx
@@ -493,17 +493,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>5 pts: Clear, specific predictive objective(s); response type (regression/classification) explicitly identified and justified; strong business/research rationale.</t>
+          <t>5 pts: Clear, specific predictive objective(s); response type (regression/classification) explicitly identified and justified; names the stakeholder and the decision the predictions support; strong business/research rationale.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>3–4 pts: Goal stated; response type identified but weakly justified; limited link to context.</t>
+          <t>3–4 pts: Goal and response type stated, but the stakeholder, the decision, or the rationale is thin; limited link to context.</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0–2 pts: Goal unclear/missing; response type unspecified; no rationale.</t>
+          <t>0–2 pts: Goal unclear/missing; response type unspecified; no link to a stakeholder's decision.</t>
         </is>
       </c>
     </row>
@@ -605,7 +605,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>14–17 pts: Appropriate simple baseline (e.g., Linear/Logistic Regression); pipeline is leakage-safe; k=5/10 CV with correct metric (RMSE/MAE/Accuracy/F1/AUC); tracks mean/variance; summarizes implications and limitations; proposes concrete next steps.</t>
+          <t>14–17 pts: Appropriate simple baseline (e.g., Linear/Logistic Regression), the incumbent any complex model must beat; pipeline is leakage-safe; k=5/10 CV (time-respecting for forecasting) with a primary metric chosen for the cost of errors; reports the fold scores with their mean and SD (no per-model confidence interval needed); summarizes implications and limitations; proposes concrete next steps.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>More Complex Model (Choice, Tuning, Paired Comparison)</t>
+          <t>Model Comparison and Champion Selection (Choice, Tuning, Paired Comparison, Rationale)</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -633,17 +633,17 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>22–25 pts: Model aligned to data/goal (RF/GBM/XGBoost/SVM/regularized GLM/NN); hyperparameter search (grid/random/Bayesian) inside proper CV; leakage controls (scaling/encoding inside folds); compared with the baseline on identical folds (same splitter and seed) using per-fold paired differences (positive favors the complex model) against a margin stated before the results; mean difference reported with an approximate 95% interval corrected for fold overlap: mean ± t × SD(differences) × √(1/k + 1/(k−1)); verdict names the outcome: worthwhile gain (interval entirely above the margin), worthwhile loss (entirely below minus the margin), practically equivalent (entirely inside ± the margin: the simpler model wins), or unresolved (anything else: the simpler model stays as a stated policy, not called equivalent); practical interpretation (effect sizes, trade-offs), plus error/confusion analysis where relevant.</t>
+          <t>22–25 pts: Model aligned to data/goal (e.g., RF/GBM/SVM/NN); tuning inside CV with leakage controls. Before comparing: primary metric, margin δ (smallest gain that would change the stakeholder's decision, with its business meaning), and candidate order (simplest first). Identical folds; per-fold differences (positive favors the challenger); interval corrected for fold overlap: mean ± t × SD(differences) × √(1/k + 1/(k−1)); outcome named: worthwhile gain (entirely above δ), worthwhile loss (entirely below −δ), practically equivalent (entirely inside ±δ), or unresolved. One champion (the baseline can win); extra complexity only on a worthwhile gain; rationale in the stakeholder's terms (what the gain means, secondary checks, runner-up, what would change the decision). Fold wins are description only; no model's own interval, interval overlap, or lower bound picks the champion; the test set is not used to select.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>13–21 pts: Plausible model; some tuning with partial documentation; CV present but thin; compares with the baseline on CV means or side-by-side intervals rather than paired per-fold differences; judges a winner or a tie by whether intervals overlap or by fold signs alone; calls the models equivalent when the interval extends past the margin; or states no margin; limited practical takeaways.</t>
+          <t>13–21 pts: Plausible model and tuning, but the comparison or decision is incomplete: folds not paired; δ missing, set after the results, or without business meaning; verdict from means, overlap, fold signs, or a model's own interval; unresolved called equivalent; or a champion without a rationale tied to the decision.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>0–12 pts: Misaligned/unspecified model; superficial/absent tuning; incorrect CV; opaque selection; no clear comparison or interpretation.</t>
+          <t>0–12 pts: Misaligned/unspecified model; superficial/absent tuning; incorrect CV; no clear comparison and no justified champion.</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>9–10 pts: Clear, scannable poster; logical flow (Intro→Methods→Results→Conclusions); legible, labeled figures/tables (titles, axes, units, legends); consistent typography/layout; code refs/appendix where appropriate; minimal grammar issues.</t>
+          <t>9–10 pts: Clear, scannable poster; logical flow (Intro→Methods→Results→Conclusions); the champion and its main reason are easy to find; legible, labeled figures/tables (titles, axes, units, legends); consistent typography/layout; code refs/appendix where appropriate; minimal grammar issues.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">

</xml_diff>

<commit_message>
fix: Make the Fall 2026 note control rubric criterion 6
The corrected paired interval is recommended, not required, this term.
Criterion 6's Exemplary level accepts notebook 08's rule applied
correctly, and the Competent deductions apply only to the rule a team
used. A disclosed after-the-fact margin is no longer listed as a
deduction. M09/M10 instructions match; points unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_final_project/2026F/rubric/Predictive_Analytics_Poster_Rubric.xlsx
+++ b/_final_project/2026F/rubric/Predictive_Analytics_Poster_Rubric.xlsx
@@ -633,12 +633,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>22–25 pts: Model aligned to data/goal (e.g., RF/GBM/SVM/NN); tuning inside CV with leakage controls. Before comparing: primary metric, margin δ (smallest gain that would change the stakeholder's decision, with its business meaning), and candidate order (simplest first). Identical folds; per-fold differences (positive favors the challenger); interval corrected for fold overlap: mean ± t × SD(differences) × √(1/k + 1/(k−1)); outcome named: worthwhile gain (entirely above δ), worthwhile loss (entirely below −δ), practically equivalent (entirely inside ±δ), or unresolved. One champion (the baseline can win); extra complexity only on a worthwhile gain; rationale in the stakeholder's terms (what the gain means, secondary checks, runner-up, what would change the decision). Fold wins are description only; no model's own interval, interval overlap, or lower bound picks the champion; the test set is not used to select.</t>
+          <t>22–25 pts: Model aligned to data/goal (e.g., RF/GBM/SVM/NN); tuning inside CV with leakage controls. Before comparing: primary metric, margin δ (smallest gain that would change the stakeholder's decision, with its business meaning), and candidate order (simplest first). Identical folds; per-fold differences (positive favors the challenger); the verdict from a rule applied correctly: notebook 08's rule (Fall 2026 note) or, recommended, the interval corrected for fold overlap, mean ± t × SD(differences) × √(1/k + 1/(k−1)), named as worthwhile gain (entirely above δ), worthwhile loss (entirely below −δ), practically equivalent (entirely inside ±δ), or unresolved. One champion (the baseline can win); extra complexity only on a worthwhile gain; rationale in the stakeholder's terms (what the gain means, secondary checks, runner-up, what would change the decision). No model's own interval, interval overlap, or lower bound picks the champion; the test set is not used to select.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>13–21 pts: Plausible model and tuning, but the comparison or decision is incomplete: folds not paired; δ missing, set after the results, or without business meaning; verdict from means, overlap, fold signs, or a model's own interval; unresolved called equivalent; or a champion without a rationale tied to the decision.</t>
+          <t>13–21 pts: Plausible model and tuning, but the comparison or decision is incomplete, or misapplies the rule the team used: folds not paired; δ missing, without business meaning, or set after the results without saying so; verdict from means alone, interval overlap, or a model's own interval; with the corrected interval, unresolved called equivalent; or a champion without a rationale tied to the decision.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">

</xml_diff>

<commit_message>
fix: Align the poster rubric and template with the published notebooks
Until the Nov 8 notebook update, criterion 6 scores notebook 08's
three-outcome paired rule against a practical margin and the champion
selection notebook 14 teaches; the corrected interval, four outcomes
and delta move out of the rubric. Criterion 5 again asks for the CV mean
with its descriptive 95% interval. The template's methodology, results
and business-implication prompts follow nb08/nb14/nb17, and the
acknowledgements box now carries a references placeholder.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_final_project/2026F/rubric/Predictive_Analytics_Poster_Rubric.xlsx
+++ b/_final_project/2026F/rubric/Predictive_Analytics_Poster_Rubric.xlsx
@@ -605,7 +605,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>14–17 pts: Appropriate simple baseline (e.g., Linear/Logistic Regression), the incumbent any complex model must beat; pipeline is leakage-safe; k=5/10 CV (time-respecting for forecasting) with a primary metric chosen for the cost of errors; reports the fold scores with their mean and SD (no per-model confidence interval needed); summarizes implications and limitations; proposes concrete next steps.</t>
+          <t>14–17 pts: Appropriate simple baseline (e.g., Linear/Logistic Regression), the reference any complex model must beat; pipeline is leakage-safe; k=5/10 CV (time-respecting for forecasting) with a primary metric chosen for the cost of errors; reports the CV mean with its SD and approximate 95% interval, labeled descriptive (notebook 08); summarizes implications and limitations; proposes concrete next steps.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -633,12 +633,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>22–25 pts: Model aligned to data/goal (e.g., RF/GBM/SVM/NN); tuning inside CV with leakage controls. Before comparing: primary metric, margin δ (smallest gain that would change the stakeholder's decision, with its business meaning), and candidate order (simplest first). Identical folds; per-fold differences (positive favors the challenger); the verdict from a rule applied correctly: notebook 08's rule (Fall 2026 note) or, recommended, the interval corrected for fold overlap, mean ± t × SD(differences) × √(1/k + 1/(k−1)), named as worthwhile gain (entirely above δ), worthwhile loss (entirely below −δ), practically equivalent (entirely inside ±δ), or unresolved. One champion (the baseline can win); extra complexity only on a worthwhile gain; rationale in the stakeholder's terms (what the gain means, secondary checks, runner-up, what would change the decision). No model's own interval, interval overlap, or lower bound picks the champion; the test set is not used to select.</t>
+          <t>22–25 pts: Model aligned to data/goal (e.g., RF/GBM/SVM/NN); tuning inside CV with leakage controls. Before comparing: the primary metric and a practical margin (the smallest gain that would change the stakeholder's decision, with its business meaning). Baseline and tuned model (and any other finalist) compared on identical folds (same splitter and seed): per-fold paired differences and their mean, with the verdict named correctly under notebook 08's rule: real difference (every fold favors the same model and the mean gap clears the margin), no winner (the sign changes across folds), or practically equivalent (same sign but under the margin, so the simpler model wins). One champion, chosen as notebook 14 teaches (the baseline can win); extra complexity only on a real difference; rationale in the stakeholder's terms (what the gain means, secondary checks, runner-up). Interval overlap does not pick the champion; the test set is not used to select.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>13–21 pts: Plausible model and tuning, but the comparison or decision is incomplete, or misapplies the rule the team used: folds not paired; δ missing, without business meaning, or set after the results without saying so; verdict from means alone, interval overlap, or a model's own interval; with the corrected interval, unresolved called equivalent; or a champion without a rationale tied to the decision.</t>
+          <t>13–21 pts: Plausible model and tuning, but the comparison or decision is incomplete or misapplied: folds not paired; margin missing, without business meaning, or set after the results without saying so; verdict from means alone or from whether two intervals overlap; fold signs that disagree read as a win; or a champion without a rationale tied to the decision.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">

</xml_diff>